<commit_message>
Release update - removed some extraneous files, hopefully from git histroy,
-update README
-updated inputs to match new interface
- Added GBC and GeneHist modules
</commit_message>
<xml_diff>
--- a/data/User_Template/user_cutoff_table.xlsx
+++ b/data/User_Template/user_cutoff_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samhamilton/editdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samhamilton/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4AC382D-3909-5B42-A558-33A6387E5C90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3492567-2E8F-0B4D-BFF7-BAD82EC24689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35480" yWindow="-5140" windowWidth="20420" windowHeight="15940" xr2:uid="{5C784FC6-2B83-B045-89F6-2FB16FF24012}"/>
+    <workbookView xWindow="35480" yWindow="-2020" windowWidth="20420" windowHeight="15940" xr2:uid="{5C784FC6-2B83-B045-89F6-2FB16FF24012}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,19 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Sequencing Depth</t>
-  </si>
-  <si>
-    <t>% of Reads After Trimming</t>
-  </si>
-  <si>
-    <t>% Uniquely Aligned Reads / Trimmed Reads</t>
-  </si>
-  <si>
-    <t>% Mapped Reads / Aligned Reads</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>% Overrep Sequences (Post-Trim)</t>
   </si>
@@ -56,28 +44,34 @@
     <t>% Adapter Content (Post-Trim)</t>
   </si>
   <si>
-    <t>% Adapter Content (Pre-Trim)</t>
-  </si>
-  <si>
-    <t>% Overrep Sequences (Pre-Trim)</t>
-  </si>
-  <si>
     <t># Detected Genes</t>
   </si>
   <si>
-    <t>Gene Body Coverage (Pval)</t>
-  </si>
-  <si>
     <t>Warn</t>
   </si>
   <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>rRNA Reads / Aligned Reads</t>
-  </si>
-  <si>
     <t>Cutoff</t>
+  </si>
+  <si>
+    <t>% Uniquely Aligned Reads</t>
+  </si>
+  <si>
+    <t>% rRNA Reads</t>
+  </si>
+  <si>
+    <t>Gene Body Coverage</t>
+  </si>
+  <si>
+    <t>% Post-Trim Reads</t>
+  </si>
+  <si>
+    <t># Sequenced Reads</t>
+  </si>
+  <si>
+    <t>% Reads Mapped To Exons</t>
   </si>
 </sst>
 </file>
@@ -133,9 +127,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -173,7 +167,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -279,7 +273,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -421,7 +415,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -429,59 +423,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DCA1397-307F-3242-9D98-CDE0DE6811C5}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="29.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="H1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="I1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>4</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>